<commit_message>
new changes final one
</commit_message>
<xml_diff>
--- a/Model Validations/Aircrafts.xlsx
+++ b/Model Validations/Aircrafts.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Important File\Crew Management\POC\Vendors\Mu Sigma\Model Output\Model Validations\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Important File\Crew Management\POC\Model Evaluation\Fixed\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{25B321F0-8BD5-4BB1-ACFF-4C9F338C8378}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D12F46F-32CE-43E8-865A-9FACEC427E32}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="19090" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Aircrafts" sheetId="1" r:id="rId1"/>
@@ -22,9 +22,6 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="210" uniqueCount="100">
   <si>
-    <t>No.</t>
-  </si>
-  <si>
     <t>Aircraft Type</t>
   </si>
   <si>
@@ -320,6 +317,9 @@
   </si>
   <si>
     <t>TMZ</t>
+  </si>
+  <si>
+    <t>Aircraft code</t>
   </si>
 </sst>
 </file>
@@ -454,7 +454,7 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table1" displayName="Table1" ref="A1:O66" totalsRowShown="0" headerRowDxfId="16" dataDxfId="15">
   <autoFilter ref="A1:O66" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}"/>
   <tableColumns count="15">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="No." dataDxfId="14"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Aircraft code" dataDxfId="14"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Aircraft Type" dataDxfId="13"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="A/C GroupCode" dataDxfId="12"/>
     <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Seat Capacity" dataDxfId="11"/>
@@ -794,7 +794,7 @@
   <dimension ref="A1:O66"/>
   <sheetFormatPr defaultColWidth="9.21875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="8.33203125" style="2" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.109375" style="2" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="16" style="2" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="18.5546875" style="2" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="17.109375" style="2" bestFit="1" customWidth="1"/>
@@ -814,60 +814,60 @@
   <sheetData>
     <row r="1" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>0</v>
+        <v>99</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
       <c r="D1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="M1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="N1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="O1" s="1" t="s">
         <v>13</v>
-      </c>
-      <c r="O1" s="1" t="s">
-        <v>14</v>
       </c>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B2" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C2" s="3" t="s">
         <v>16</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>17</v>
       </c>
       <c r="D2" s="4">
         <v>15</v>
@@ -908,13 +908,13 @@
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C3" s="3" t="s">
         <v>18</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>19</v>
       </c>
       <c r="D3" s="4">
         <v>16</v>
@@ -955,13 +955,13 @@
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B4" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="C4" s="3" t="s">
         <v>21</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>22</v>
       </c>
       <c r="D4" s="4">
         <v>15</v>
@@ -1002,13 +1002,13 @@
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C5" s="3" t="s">
         <v>23</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>24</v>
       </c>
       <c r="D5" s="4">
         <v>15</v>
@@ -1049,13 +1049,13 @@
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A6" s="3" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D6" s="4">
         <v>15</v>
@@ -1096,13 +1096,13 @@
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A7" s="3" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B7" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="C7" s="3" t="s">
         <v>21</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>22</v>
       </c>
       <c r="D7" s="4">
         <v>15</v>
@@ -1143,13 +1143,13 @@
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A8" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="C8" s="3" t="s">
         <v>27</v>
-      </c>
-      <c r="B8" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="C8" s="3" t="s">
-        <v>28</v>
       </c>
       <c r="D8" s="4">
         <v>15</v>
@@ -1190,13 +1190,13 @@
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A9" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C9" s="3" t="s">
         <v>29</v>
-      </c>
-      <c r="B9" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="C9" s="3" t="s">
-        <v>30</v>
       </c>
       <c r="D9" s="4">
         <v>9</v>
@@ -1237,13 +1237,13 @@
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A10" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="B10" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="B10" s="3" t="s">
+      <c r="C10" s="3" t="s">
         <v>32</v>
-      </c>
-      <c r="C10" s="3" t="s">
-        <v>33</v>
       </c>
       <c r="D10" s="4">
         <v>10</v>
@@ -1284,13 +1284,13 @@
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A11" s="3" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D11" s="4">
         <v>16</v>
@@ -1331,13 +1331,13 @@
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A12" s="3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D12" s="4">
         <v>15</v>
@@ -1378,13 +1378,13 @@
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A13" s="3" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D13" s="4">
         <v>15</v>
@@ -1425,13 +1425,13 @@
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A14" s="3" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D14" s="4">
         <v>15</v>
@@ -1472,13 +1472,13 @@
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A15" s="3" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D15" s="4">
         <v>16</v>
@@ -1519,13 +1519,13 @@
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A16" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="C16" s="3" t="s">
         <v>39</v>
-      </c>
-      <c r="B16" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="C16" s="3" t="s">
-        <v>40</v>
       </c>
       <c r="D16" s="4">
         <v>15</v>
@@ -1566,13 +1566,13 @@
     </row>
     <row r="17" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A17" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C17" s="3" t="s">
         <v>41</v>
-      </c>
-      <c r="B17" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="C17" s="3" t="s">
-        <v>42</v>
       </c>
       <c r="D17" s="4">
         <v>8</v>
@@ -1613,13 +1613,13 @@
     </row>
     <row r="18" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A18" s="3" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D18" s="4">
         <v>15</v>
@@ -1660,13 +1660,13 @@
     </row>
     <row r="19" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A19" s="3" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D19" s="4">
         <v>15</v>
@@ -1707,13 +1707,13 @@
     </row>
     <row r="20" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A20" s="3" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D20" s="4">
         <v>15</v>
@@ -1754,13 +1754,13 @@
     </row>
     <row r="21" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A21" s="3" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B21" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C21" s="3" t="s">
         <v>16</v>
-      </c>
-      <c r="C21" s="3" t="s">
-        <v>17</v>
       </c>
       <c r="D21" s="4">
         <v>15</v>
@@ -1801,13 +1801,13 @@
     </row>
     <row r="22" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A22" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="B22" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="B22" s="3" t="s">
+      <c r="C22" s="3" t="s">
         <v>48</v>
-      </c>
-      <c r="C22" s="3" t="s">
-        <v>49</v>
       </c>
       <c r="D22" s="4">
         <v>15</v>
@@ -1848,13 +1848,13 @@
     </row>
     <row r="23" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A23" s="3" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C23" s="3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D23" s="4">
         <v>15</v>
@@ -1895,13 +1895,13 @@
     </row>
     <row r="24" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A24" s="3" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C24" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D24" s="4">
         <v>15</v>
@@ -1942,13 +1942,13 @@
     </row>
     <row r="25" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A25" s="3" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C25" s="3" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D25" s="4">
         <v>15</v>
@@ -1989,13 +1989,13 @@
     </row>
     <row r="26" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A26" s="3" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C26" s="3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D26" s="4">
         <v>15</v>
@@ -2036,13 +2036,13 @@
     </row>
     <row r="27" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A27" s="3" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C27" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D27" s="4">
         <v>15</v>
@@ -2083,13 +2083,13 @@
     </row>
     <row r="28" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A28" s="3" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C28" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D28" s="4">
         <v>15</v>
@@ -2130,13 +2130,13 @@
     </row>
     <row r="29" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A29" s="3" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C29" s="3" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D29" s="4">
         <v>8</v>
@@ -2177,13 +2177,13 @@
     </row>
     <row r="30" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A30" s="3" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C30" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D30" s="4">
         <v>15</v>
@@ -2224,13 +2224,13 @@
     </row>
     <row r="31" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A31" s="3" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C31" s="3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D31" s="4">
         <v>15</v>
@@ -2271,13 +2271,13 @@
     </row>
     <row r="32" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A32" s="3" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C32" s="3" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D32" s="4">
         <v>15</v>
@@ -2318,13 +2318,13 @@
     </row>
     <row r="33" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A33" s="3" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B33" s="3" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C33" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D33" s="4">
         <v>15</v>
@@ -2365,13 +2365,13 @@
     </row>
     <row r="34" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A34" s="3" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B34" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="C34" s="3" t="s">
         <v>21</v>
-      </c>
-      <c r="C34" s="3" t="s">
-        <v>22</v>
       </c>
       <c r="D34" s="4">
         <v>15</v>
@@ -2412,13 +2412,13 @@
     </row>
     <row r="35" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A35" s="3" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B35" s="3" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C35" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D35" s="4">
         <v>15</v>
@@ -2459,13 +2459,13 @@
     </row>
     <row r="36" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A36" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="B36" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="B36" s="3" t="s">
-        <v>64</v>
-      </c>
       <c r="C36" s="3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D36" s="4">
         <v>15</v>
@@ -2506,13 +2506,13 @@
     </row>
     <row r="37" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A37" s="3" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B37" s="3" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C37" s="3" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D37" s="4">
         <v>15</v>
@@ -2553,13 +2553,13 @@
     </row>
     <row r="38" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A38" s="3" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B38" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C38" s="3" t="s">
         <v>16</v>
-      </c>
-      <c r="C38" s="3" t="s">
-        <v>17</v>
       </c>
       <c r="D38" s="4">
         <v>12</v>
@@ -2600,13 +2600,13 @@
     </row>
     <row r="39" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A39" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="B39" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="B39" s="3" t="s">
-        <v>68</v>
-      </c>
       <c r="C39" s="3" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D39" s="4">
         <v>10</v>
@@ -2647,13 +2647,13 @@
     </row>
     <row r="40" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A40" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="B40" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="B40" s="3" t="s">
-        <v>70</v>
-      </c>
       <c r="C40" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D40" s="4">
         <v>15</v>
@@ -2694,13 +2694,13 @@
     </row>
     <row r="41" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A41" s="3" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B41" s="3" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C41" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D41" s="4">
         <v>15</v>
@@ -2741,13 +2741,13 @@
     </row>
     <row r="42" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A42" s="3" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B42" s="3" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C42" s="3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D42" s="4">
         <v>15</v>
@@ -2788,13 +2788,13 @@
     </row>
     <row r="43" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A43" s="3" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B43" s="3" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C43" s="3" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D43" s="4">
         <v>15</v>
@@ -2835,13 +2835,13 @@
     </row>
     <row r="44" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A44" s="3" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B44" s="3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C44" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D44" s="4">
         <v>15</v>
@@ -2882,13 +2882,13 @@
     </row>
     <row r="45" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A45" s="3" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B45" s="3" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C45" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D45" s="4">
         <v>16</v>
@@ -2929,13 +2929,13 @@
     </row>
     <row r="46" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A46" s="3" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B46" s="3" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C46" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D46" s="4">
         <v>15</v>
@@ -2976,13 +2976,13 @@
     </row>
     <row r="47" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A47" s="3" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B47" s="3" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C47" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D47" s="4">
         <v>15</v>
@@ -3023,13 +3023,13 @@
     </row>
     <row r="48" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A48" s="3" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B48" s="3" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C48" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D48" s="4">
         <v>15</v>
@@ -3070,13 +3070,13 @@
     </row>
     <row r="49" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A49" s="3" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B49" s="3" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C49" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D49" s="4">
         <v>15</v>
@@ -3117,13 +3117,13 @@
     </row>
     <row r="50" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A50" s="3" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B50" s="3" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C50" s="3" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D50" s="4">
         <v>15</v>
@@ -3164,13 +3164,13 @@
     </row>
     <row r="51" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A51" s="3" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B51" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C51" s="3" t="s">
         <v>16</v>
-      </c>
-      <c r="C51" s="3" t="s">
-        <v>17</v>
       </c>
       <c r="D51" s="4">
         <v>8</v>
@@ -3211,13 +3211,13 @@
     </row>
     <row r="52" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A52" s="3" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B52" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="C52" s="3" t="s">
         <v>21</v>
-      </c>
-      <c r="C52" s="3" t="s">
-        <v>22</v>
       </c>
       <c r="D52" s="4">
         <v>15</v>
@@ -3258,13 +3258,13 @@
     </row>
     <row r="53" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A53" s="3" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B53" s="3" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C53" s="3" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D53" s="4">
         <v>15</v>
@@ -3305,13 +3305,13 @@
     </row>
     <row r="54" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A54" s="3" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B54" s="3" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C54" s="3" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D54" s="4">
         <v>15</v>
@@ -3352,13 +3352,13 @@
     </row>
     <row r="55" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A55" s="3" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B55" s="3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C55" s="3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D55" s="4">
         <v>15</v>
@@ -3399,13 +3399,13 @@
     </row>
     <row r="56" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A56" s="3" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B56" s="3" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C56" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D56" s="4">
         <v>15</v>
@@ -3446,13 +3446,13 @@
     </row>
     <row r="57" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A57" s="3" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B57" s="3" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C57" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D57" s="4">
         <v>15</v>
@@ -3493,13 +3493,13 @@
     </row>
     <row r="58" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A58" s="3" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B58" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C58" s="3" t="s">
         <v>16</v>
-      </c>
-      <c r="C58" s="3" t="s">
-        <v>17</v>
       </c>
       <c r="D58" s="4">
         <v>15</v>
@@ -3540,13 +3540,13 @@
     </row>
     <row r="59" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A59" s="3" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B59" s="3" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C59" s="3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D59" s="4">
         <v>15</v>
@@ -3587,13 +3587,13 @@
     </row>
     <row r="60" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A60" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="B60" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C60" s="3" t="s">
         <v>90</v>
-      </c>
-      <c r="B60" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="C60" s="3" t="s">
-        <v>91</v>
       </c>
       <c r="D60" s="4">
         <v>9</v>
@@ -3634,13 +3634,13 @@
     </row>
     <row r="61" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A61" s="3" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B61" s="3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C61" s="3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D61" s="4">
         <v>15</v>
@@ -3681,13 +3681,13 @@
     </row>
     <row r="62" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A62" s="3" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B62" s="3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C62" s="3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D62" s="4">
         <v>15</v>
@@ -3728,13 +3728,13 @@
     </row>
     <row r="63" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A63" s="3" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B63" s="3" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C63" s="3" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D63" s="4">
         <v>15</v>
@@ -3775,13 +3775,13 @@
     </row>
     <row r="64" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A64" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="B64" s="3" t="s">
         <v>95</v>
       </c>
-      <c r="B64" s="3" t="s">
+      <c r="C64" s="3" t="s">
         <v>96</v>
-      </c>
-      <c r="C64" s="3" t="s">
-        <v>97</v>
       </c>
       <c r="D64" s="4">
         <v>15</v>
@@ -3822,13 +3822,13 @@
     </row>
     <row r="65" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A65" s="3" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B65" s="3" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C65" s="3" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D65" s="4">
         <v>15</v>
@@ -3869,13 +3869,13 @@
     </row>
     <row r="66" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A66" s="3" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B66" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="C66" s="3" t="s">
         <v>96</v>
-      </c>
-      <c r="C66" s="3" t="s">
-        <v>97</v>
       </c>
       <c r="D66" s="4">
         <v>15</v>

</xml_diff>